<commit_message>
Update schedule file: Y4_B2526_General_&_Special_Internal_1_A1_schedule.xlsx
</commit_message>
<xml_diff>
--- a/modules_schedules/Y4_B2526_General_&_Special_Internal_1_A1_schedule.xlsx
+++ b/modules_schedules/Y4_B2526_General_&_Special_Internal_1_A1_schedule.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G249"/>
+  <dimension ref="A1:G245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -670,12 +670,12 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>04/04/2026</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -705,12 +705,12 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -740,12 +740,12 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -775,12 +775,12 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -810,12 +810,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -840,17 +840,17 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -880,12 +880,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -950,12 +950,12 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -985,12 +985,12 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1055,12 +1055,12 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1125,12 +1125,12 @@
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1160,12 +1160,12 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1190,17 +1190,17 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1230,12 +1230,12 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1300,12 +1300,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -1365,17 +1365,17 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1405,12 +1405,12 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -1440,12 +1440,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1475,12 +1475,12 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>11/03/2026</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -1510,12 +1510,12 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1545,12 +1545,12 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>12/03/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -1580,12 +1580,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
@@ -1615,12 +1615,12 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="F33" s="8" t="inlineStr">
@@ -1650,12 +1650,12 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
@@ -1685,12 +1685,12 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -1715,17 +1715,17 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>22/02/2026</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
@@ -1755,12 +1755,12 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>22/02/2026</t>
+          <t>23/02/2026</t>
         </is>
       </c>
       <c r="F37" s="8" t="inlineStr">
@@ -1790,12 +1790,12 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
@@ -1825,12 +1825,12 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -1895,12 +1895,12 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
@@ -1965,12 +1965,12 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="F43" s="8" t="inlineStr">
@@ -2000,12 +2000,12 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>03/03/2026</t>
+          <t>04/03/2026</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
@@ -2035,12 +2035,12 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>05/03/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
@@ -2105,12 +2105,12 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -2140,12 +2140,12 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -2210,12 +2210,12 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -2235,22 +2235,22 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>A1A</t>
+          <t>A1B</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>tropical medicine</t>
+          <t>cardiology</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -2280,12 +2280,12 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -2315,12 +2315,12 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -2350,12 +2350,12 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
@@ -2385,12 +2385,12 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>14/03/2026</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -2420,12 +2420,12 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
@@ -2455,12 +2455,12 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>14/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="F57" s="8" t="inlineStr">
@@ -2490,12 +2490,12 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
@@ -2525,12 +2525,12 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -2555,17 +2555,17 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -2590,17 +2590,17 @@
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -2630,12 +2630,12 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
@@ -2665,12 +2665,12 @@
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -2700,12 +2700,12 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -2735,12 +2735,12 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -2770,12 +2770,12 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
@@ -2805,12 +2805,12 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -2840,12 +2840,12 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
@@ -2875,12 +2875,12 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="F69" s="8" t="inlineStr">
@@ -2905,17 +2905,17 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
@@ -2940,17 +2940,17 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="F71" s="8" t="inlineStr">
@@ -2980,12 +2980,12 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
@@ -3015,12 +3015,12 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -3050,12 +3050,12 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
@@ -3080,17 +3080,17 @@
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>22/02/2026</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
@@ -3115,17 +3115,17 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>23/02/2026</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
@@ -3155,12 +3155,12 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>22/02/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
@@ -3190,12 +3190,12 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
@@ -3225,12 +3225,12 @@
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -3260,12 +3260,12 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
@@ -3295,12 +3295,12 @@
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="F81" s="8" t="inlineStr">
@@ -3330,12 +3330,12 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="F82" s="4" t="inlineStr">
@@ -3365,12 +3365,12 @@
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>04/03/2026</t>
         </is>
       </c>
       <c r="F83" s="8" t="inlineStr">
@@ -3400,12 +3400,12 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>03/03/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
@@ -3430,17 +3430,17 @@
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="F85" s="8" t="inlineStr">
@@ -3465,17 +3465,17 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>05/03/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -3505,12 +3505,12 @@
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="F87" s="8" t="inlineStr">
@@ -3540,12 +3540,12 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="F88" s="4" t="inlineStr">
@@ -3575,12 +3575,12 @@
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="F89" s="8" t="inlineStr">
@@ -3610,12 +3610,12 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
@@ -3645,12 +3645,12 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="F91" s="8" t="inlineStr">
@@ -3680,12 +3680,12 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="F93" s="8" t="inlineStr">
@@ -3750,12 +3750,12 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="F94" s="4" t="inlineStr">
@@ -3780,17 +3780,17 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="F95" s="8" t="inlineStr">
@@ -3815,17 +3815,17 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="F96" s="4" t="inlineStr">
@@ -3855,12 +3855,12 @@
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="F97" s="8" t="inlineStr">
@@ -3890,12 +3890,12 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
@@ -3915,22 +3915,22 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>A1B</t>
+          <t>A1C</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>tropical medicine</t>
+          <t>cardiology</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>21/02/2026</t>
         </is>
       </c>
       <c r="F99" s="8" t="inlineStr">
@@ -3950,22 +3950,22 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>A1B</t>
+          <t>A1C</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>tropical medicine</t>
+          <t>cardiology</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>22/02/2026</t>
         </is>
       </c>
       <c r="F100" s="4" t="inlineStr">
@@ -3995,12 +3995,12 @@
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>21/02/2026</t>
+          <t>23/02/2026</t>
         </is>
       </c>
       <c r="F101" s="8" t="inlineStr">
@@ -4030,12 +4030,12 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>22/02/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="F102" s="4" t="inlineStr">
@@ -4065,12 +4065,12 @@
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>28/02/2026</t>
         </is>
       </c>
       <c r="F103" s="8" t="inlineStr">
@@ -4100,12 +4100,12 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="F104" s="4" t="inlineStr">
@@ -4135,12 +4135,12 @@
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="F105" s="8" t="inlineStr">
@@ -4170,12 +4170,12 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="F106" s="4" t="inlineStr">
@@ -4205,12 +4205,12 @@
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>04/03/2026</t>
         </is>
       </c>
       <c r="F107" s="8" t="inlineStr">
@@ -4235,17 +4235,17 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>03/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="F108" s="4" t="inlineStr">
@@ -4270,17 +4270,17 @@
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="F109" s="8" t="inlineStr">
@@ -4310,12 +4310,12 @@
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="F110" s="4" t="inlineStr">
@@ -4345,12 +4345,12 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>11/03/2026</t>
         </is>
       </c>
       <c r="F111" s="8" t="inlineStr">
@@ -4380,12 +4380,12 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E112" s="3" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="F112" s="4" t="inlineStr">
@@ -4415,12 +4415,12 @@
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="F113" s="8" t="inlineStr">
@@ -4450,12 +4450,12 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E114" s="3" t="inlineStr">
         <is>
-          <t>12/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="F114" s="4" t="inlineStr">
@@ -4485,12 +4485,12 @@
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="F115" s="8" t="inlineStr">
@@ -4520,12 +4520,12 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E116" s="3" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F116" s="4" t="inlineStr">
@@ -4555,12 +4555,12 @@
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F117" s="8" t="inlineStr">
@@ -4585,17 +4585,17 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E118" s="3" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="F118" s="4" t="inlineStr">
@@ -4620,17 +4620,17 @@
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="F119" s="8" t="inlineStr">
@@ -4660,12 +4660,12 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="F120" s="4" t="inlineStr">
@@ -4695,12 +4695,12 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="F121" s="8" t="inlineStr">
@@ -4730,12 +4730,12 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E122" s="3" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="F122" s="4" t="inlineStr">
@@ -4760,17 +4760,17 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="F123" s="8" t="inlineStr">
@@ -4795,17 +4795,17 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="F124" s="4" t="inlineStr">
@@ -4835,12 +4835,12 @@
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="F125" s="8" t="inlineStr">
@@ -4870,12 +4870,12 @@
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="F126" s="4" t="inlineStr">
@@ -4905,12 +4905,12 @@
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="F127" s="8" t="inlineStr">
@@ -4940,12 +4940,12 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="F128" s="4" t="inlineStr">
@@ -4975,12 +4975,12 @@
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="F129" s="8" t="inlineStr">
@@ -5010,12 +5010,12 @@
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="F130" s="4" t="inlineStr">
@@ -5045,12 +5045,12 @@
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="F131" s="8" t="inlineStr">
@@ -5080,12 +5080,12 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="F132" s="4" t="inlineStr">
@@ -5110,17 +5110,17 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="F133" s="8" t="inlineStr">
@@ -5145,17 +5145,17 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="F134" s="4" t="inlineStr">
@@ -5185,12 +5185,12 @@
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="F135" s="8" t="inlineStr">
@@ -5220,12 +5220,12 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="F136" s="4" t="inlineStr">
@@ -5255,12 +5255,12 @@
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="F137" s="8" t="inlineStr">
@@ -5290,12 +5290,12 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="F138" s="4" t="inlineStr">
@@ -5325,12 +5325,12 @@
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="F139" s="8" t="inlineStr">
@@ -5360,12 +5360,12 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="F140" s="4" t="inlineStr">
@@ -5395,12 +5395,12 @@
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="F141" s="8" t="inlineStr">
@@ -5430,12 +5430,12 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="F142" s="4" t="inlineStr">
@@ -5460,17 +5460,17 @@
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="F143" s="8" t="inlineStr">
@@ -5495,17 +5495,17 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="F144" s="4" t="inlineStr">
@@ -5535,12 +5535,12 @@
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="F145" s="8" t="inlineStr">
@@ -5570,12 +5570,12 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F146" s="4" t="inlineStr">
@@ -5605,12 +5605,12 @@
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="F147" s="8" t="inlineStr">
@@ -5630,22 +5630,22 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>A1C</t>
+          <t>A1D</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>tropical medicine</t>
+          <t>cardiology</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="F148" s="4" t="inlineStr">
@@ -5665,22 +5665,22 @@
       </c>
       <c r="B149" s="6" t="inlineStr">
         <is>
-          <t>A1C</t>
+          <t>A1D</t>
         </is>
       </c>
       <c r="C149" s="6" t="inlineStr">
         <is>
-          <t>tropical medicine</t>
+          <t>cardiology</t>
         </is>
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="F149" s="8" t="inlineStr">
@@ -5710,12 +5710,12 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="F150" s="4" t="inlineStr">
@@ -5745,12 +5745,12 @@
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="F151" s="8" t="inlineStr">
@@ -5780,12 +5780,12 @@
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="F152" s="4" t="inlineStr">
@@ -5815,12 +5815,12 @@
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="F153" s="8" t="inlineStr">
@@ -5850,12 +5850,12 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="F154" s="4" t="inlineStr">
@@ -5885,12 +5885,12 @@
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="F155" s="8" t="inlineStr">
@@ -5920,12 +5920,12 @@
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="F156" s="4" t="inlineStr">
@@ -5950,17 +5950,17 @@
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>22/02/2026</t>
         </is>
       </c>
       <c r="F157" s="8" t="inlineStr">
@@ -5985,17 +5985,17 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E158" s="3" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>23/02/2026</t>
         </is>
       </c>
       <c r="F158" s="4" t="inlineStr">
@@ -6020,17 +6020,17 @@
       </c>
       <c r="C159" s="6" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="F159" s="8" t="inlineStr">
@@ -6060,12 +6060,12 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
-          <t>22/02/2026</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="F160" s="4" t="inlineStr">
@@ -6095,12 +6095,12 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F161" s="8" t="inlineStr">
@@ -6130,12 +6130,12 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="F162" s="4" t="inlineStr">
@@ -6165,12 +6165,12 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="F163" s="8" t="inlineStr">
@@ -6200,12 +6200,12 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="F164" s="4" t="inlineStr">
@@ -6235,12 +6235,12 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>04/03/2026</t>
         </is>
       </c>
       <c r="F165" s="8" t="inlineStr">
@@ -6270,12 +6270,12 @@
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E166" s="3" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="F166" s="4" t="inlineStr">
@@ -6300,17 +6300,17 @@
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>03/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="F167" s="8" t="inlineStr">
@@ -6335,17 +6335,17 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
-          <t>04/03/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="F168" s="4" t="inlineStr">
@@ -6370,17 +6370,17 @@
       </c>
       <c r="C169" s="6" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>05/03/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="F169" s="8" t="inlineStr">
@@ -6410,12 +6410,12 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E170" s="3" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>11/03/2026</t>
         </is>
       </c>
       <c r="F170" s="4" t="inlineStr">
@@ -6445,12 +6445,12 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="F171" s="8" t="inlineStr">
@@ -6475,17 +6475,17 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="F172" s="4" t="inlineStr">
@@ -6510,17 +6510,17 @@
       </c>
       <c r="C173" s="6" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="F173" s="8" t="inlineStr">
@@ -6545,17 +6545,17 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>12/03/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="F174" s="4" t="inlineStr">
@@ -6585,12 +6585,12 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="F175" s="8" t="inlineStr">
@@ -6620,12 +6620,12 @@
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E176" s="3" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="F176" s="4" t="inlineStr">
@@ -6655,12 +6655,12 @@
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="F177" s="8" t="inlineStr">
@@ -6690,12 +6690,12 @@
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="F178" s="4" t="inlineStr">
@@ -6725,12 +6725,12 @@
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="F179" s="8" t="inlineStr">
@@ -6760,12 +6760,12 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="F180" s="4" t="inlineStr">
@@ -6795,12 +6795,12 @@
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="F181" s="8" t="inlineStr">
@@ -6825,17 +6825,17 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="F182" s="4" t="inlineStr">
@@ -6860,17 +6860,17 @@
       </c>
       <c r="C183" s="6" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="F183" s="8" t="inlineStr">
@@ -6895,17 +6895,17 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="F184" s="4" t="inlineStr">
@@ -6935,12 +6935,12 @@
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="F185" s="8" t="inlineStr">
@@ -6970,12 +6970,12 @@
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="F186" s="4" t="inlineStr">
@@ -7005,12 +7005,12 @@
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="F187" s="8" t="inlineStr">
@@ -7040,12 +7040,12 @@
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="F188" s="4" t="inlineStr">
@@ -7075,12 +7075,12 @@
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="F189" s="8" t="inlineStr">
@@ -7110,12 +7110,12 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F190" s="4" t="inlineStr">
@@ -7145,12 +7145,12 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="F191" s="8" t="inlineStr">
@@ -7175,17 +7175,17 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="F192" s="4" t="inlineStr">
@@ -7210,17 +7210,17 @@
       </c>
       <c r="C193" s="6" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="F193" s="8" t="inlineStr">
@@ -7245,17 +7245,17 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="F194" s="4" t="inlineStr">
@@ -7285,12 +7285,12 @@
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F195" s="8" t="inlineStr">
@@ -7320,12 +7320,12 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E196" s="3" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F196" s="4" t="inlineStr">
@@ -7345,22 +7345,22 @@
       </c>
       <c r="B197" s="6" t="inlineStr">
         <is>
-          <t>A1D</t>
+          <t>A1E</t>
         </is>
       </c>
       <c r="C197" s="6" t="inlineStr">
         <is>
-          <t>tropical medicine</t>
+          <t>cardiology</t>
         </is>
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="F197" s="8" t="inlineStr">
@@ -7380,22 +7380,22 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>A1D</t>
+          <t>A1E</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>tropical medicine</t>
+          <t>cardiology</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E198" s="3" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="F198" s="4" t="inlineStr">
@@ -7415,22 +7415,22 @@
       </c>
       <c r="B199" s="6" t="inlineStr">
         <is>
-          <t>A1D</t>
+          <t>A1E</t>
         </is>
       </c>
       <c r="C199" s="6" t="inlineStr">
         <is>
-          <t>tropical medicine</t>
+          <t>cardiology</t>
         </is>
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="F199" s="8" t="inlineStr">
@@ -7460,12 +7460,12 @@
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E200" s="3" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="F200" s="4" t="inlineStr">
@@ -7495,12 +7495,12 @@
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E201" s="7" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="F201" s="8" t="inlineStr">
@@ -7530,12 +7530,12 @@
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E202" s="3" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="F202" s="4" t="inlineStr">
@@ -7565,12 +7565,12 @@
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="F203" s="8" t="inlineStr">
@@ -7600,12 +7600,12 @@
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E204" s="3" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="F204" s="4" t="inlineStr">
@@ -7635,12 +7635,12 @@
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E205" s="7" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="F205" s="8" t="inlineStr">
@@ -7665,17 +7665,17 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E206" s="3" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="F206" s="4" t="inlineStr">
@@ -7700,17 +7700,17 @@
       </c>
       <c r="C207" s="6" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E207" s="7" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="F207" s="8" t="inlineStr">
@@ -7735,17 +7735,17 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E208" s="3" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="F208" s="4" t="inlineStr">
@@ -7770,17 +7770,17 @@
       </c>
       <c r="C209" s="6" t="inlineStr">
         <is>
-          <t>cardiology</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E209" s="7" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="F209" s="8" t="inlineStr">
@@ -7810,12 +7810,12 @@
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E210" s="3" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="F210" s="4" t="inlineStr">
@@ -7845,12 +7845,12 @@
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E211" s="7" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="F211" s="8" t="inlineStr">
@@ -7880,12 +7880,12 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E212" s="3" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="F212" s="4" t="inlineStr">
@@ -7915,12 +7915,12 @@
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="F213" s="8" t="inlineStr">
@@ -7950,12 +7950,12 @@
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E214" s="3" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="F214" s="4" t="inlineStr">
@@ -7985,12 +7985,12 @@
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="F215" s="8" t="inlineStr">
@@ -8015,17 +8015,17 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E216" s="3" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>22/02/2026</t>
         </is>
       </c>
       <c r="F216" s="4" t="inlineStr">
@@ -8050,17 +8050,17 @@
       </c>
       <c r="C217" s="6" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>23/02/2026</t>
         </is>
       </c>
       <c r="F217" s="8" t="inlineStr">
@@ -8085,17 +8085,17 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E218" s="3" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="F218" s="4" t="inlineStr">
@@ -8120,17 +8120,17 @@
       </c>
       <c r="C219" s="6" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>dermatology</t>
         </is>
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>25/02/2026</t>
         </is>
       </c>
       <c r="F219" s="8" t="inlineStr">
@@ -8160,12 +8160,12 @@
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E220" s="3" t="inlineStr">
         <is>
-          <t>22/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="F220" s="4" t="inlineStr">
@@ -8190,17 +8190,17 @@
       </c>
       <c r="C221" s="6" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E221" s="7" t="inlineStr">
         <is>
-          <t>23/02/2026</t>
+          <t>29/03/2026</t>
         </is>
       </c>
       <c r="F221" s="8" t="inlineStr">
@@ -8225,17 +8225,17 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E222" s="3" t="inlineStr">
         <is>
-          <t>24/02/2026</t>
+          <t>30/03/2026</t>
         </is>
       </c>
       <c r="F222" s="4" t="inlineStr">
@@ -8260,17 +8260,17 @@
       </c>
       <c r="C223" s="6" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E223" s="7" t="inlineStr">
         <is>
-          <t>25/02/2026</t>
+          <t>31/03/2026</t>
         </is>
       </c>
       <c r="F223" s="8" t="inlineStr">
@@ -8295,17 +8295,17 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>dermatology</t>
+          <t>immunology/haematology</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E224" s="3" t="inlineStr">
         <is>
-          <t>26/02/2026</t>
+          <t>01/04/2026</t>
         </is>
       </c>
       <c r="F224" s="4" t="inlineStr">
@@ -8335,12 +8335,12 @@
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E225" s="7" t="inlineStr">
         <is>
-          <t>29/03/2026</t>
+          <t>02/04/2026</t>
         </is>
       </c>
       <c r="F225" s="8" t="inlineStr">
@@ -8370,12 +8370,12 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E226" s="3" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="F226" s="4" t="inlineStr">
@@ -8405,12 +8405,12 @@
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E227" s="7" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="F227" s="8" t="inlineStr">
@@ -8440,12 +8440,12 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E228" s="3" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="F228" s="4" t="inlineStr">
@@ -8475,12 +8475,12 @@
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F229" s="8" t="inlineStr">
@@ -8510,12 +8510,12 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E230" s="3" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="F230" s="4" t="inlineStr">
@@ -8540,17 +8540,17 @@
       </c>
       <c r="C231" s="6" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E231" s="7" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="F231" s="8" t="inlineStr">
@@ -8575,17 +8575,17 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E232" s="3" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>09/03/2026</t>
         </is>
       </c>
       <c r="F232" s="4" t="inlineStr">
@@ -8610,17 +8610,17 @@
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E233" s="7" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="F233" s="8" t="inlineStr">
@@ -8645,17 +8645,17 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>immunology/haematology</t>
+          <t>psychiatry</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E234" s="3" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>11/03/2026</t>
         </is>
       </c>
       <c r="F234" s="4" t="inlineStr">
@@ -8685,12 +8685,12 @@
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>08/03/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="F235" s="8" t="inlineStr">
@@ -8720,12 +8720,12 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E236" s="3" t="inlineStr">
         <is>
-          <t>09/03/2026</t>
+          <t>15/03/2026</t>
         </is>
       </c>
       <c r="F236" s="4" t="inlineStr">
@@ -8755,12 +8755,12 @@
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="E237" s="7" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>16/03/2026</t>
         </is>
       </c>
       <c r="F237" s="8" t="inlineStr">
@@ -8790,12 +8790,12 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E238" s="3" t="inlineStr">
         <is>
-          <t>11/03/2026</t>
+          <t>17/03/2026</t>
         </is>
       </c>
       <c r="F238" s="4" t="inlineStr">
@@ -8825,12 +8825,12 @@
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E239" s="7" t="inlineStr">
         <is>
-          <t>12/03/2026</t>
+          <t>18/03/2026</t>
         </is>
       </c>
       <c r="F239" s="8" t="inlineStr">
@@ -8860,12 +8860,12 @@
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E240" s="3" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>19/03/2026</t>
         </is>
       </c>
       <c r="F240" s="4" t="inlineStr">
@@ -8890,17 +8890,17 @@
       </c>
       <c r="C241" s="6" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E241" s="7" t="inlineStr">
         <is>
-          <t>16/03/2026</t>
+          <t>01/03/2026</t>
         </is>
       </c>
       <c r="F241" s="8" t="inlineStr">
@@ -8925,17 +8925,17 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E242" s="3" t="inlineStr">
         <is>
-          <t>17/03/2026</t>
+          <t>02/03/2026</t>
         </is>
       </c>
       <c r="F242" s="4" t="inlineStr">
@@ -8960,17 +8960,17 @@
       </c>
       <c r="C243" s="6" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D243" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E243" s="7" t="inlineStr">
         <is>
-          <t>18/03/2026</t>
+          <t>03/03/2026</t>
         </is>
       </c>
       <c r="F243" s="8" t="inlineStr">
@@ -8995,17 +8995,17 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>psychiatry</t>
+          <t>tropical medicine</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E244" s="3" t="inlineStr">
         <is>
-          <t>19/03/2026</t>
+          <t>04/03/2026</t>
         </is>
       </c>
       <c r="F244" s="4" t="inlineStr">
@@ -9035,12 +9035,12 @@
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>05/03/2026</t>
         </is>
       </c>
       <c r="F245" s="8" t="inlineStr">
@@ -9049,146 +9049,6 @@
         </is>
       </c>
       <c r="G245" s="9" t="n">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B246" s="2" t="inlineStr">
-        <is>
-          <t>A1E</t>
-        </is>
-      </c>
-      <c r="C246" s="2" t="inlineStr">
-        <is>
-          <t>tropical medicine</t>
-        </is>
-      </c>
-      <c r="D246" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E246" s="3" t="inlineStr">
-        <is>
-          <t>02/03/2026</t>
-        </is>
-      </c>
-      <c r="F246" s="4" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G246" s="5" t="n">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B247" s="6" t="inlineStr">
-        <is>
-          <t>A1E</t>
-        </is>
-      </c>
-      <c r="C247" s="6" t="inlineStr">
-        <is>
-          <t>tropical medicine</t>
-        </is>
-      </c>
-      <c r="D247" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E247" s="7" t="inlineStr">
-        <is>
-          <t>03/03/2026</t>
-        </is>
-      </c>
-      <c r="F247" s="8" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G247" s="9" t="n">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="2" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B248" s="2" t="inlineStr">
-        <is>
-          <t>A1E</t>
-        </is>
-      </c>
-      <c r="C248" s="2" t="inlineStr">
-        <is>
-          <t>tropical medicine</t>
-        </is>
-      </c>
-      <c r="D248" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E248" s="3" t="inlineStr">
-        <is>
-          <t>04/03/2026</t>
-        </is>
-      </c>
-      <c r="F248" s="4" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G248" s="5" t="n">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" s="6" t="inlineStr">
-        <is>
-          <t>Year 4</t>
-        </is>
-      </c>
-      <c r="B249" s="6" t="inlineStr">
-        <is>
-          <t>A1E</t>
-        </is>
-      </c>
-      <c r="C249" s="6" t="inlineStr">
-        <is>
-          <t>tropical medicine</t>
-        </is>
-      </c>
-      <c r="D249" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E249" s="7" t="inlineStr">
-        <is>
-          <t>05/03/2026</t>
-        </is>
-      </c>
-      <c r="F249" s="8" t="inlineStr">
-        <is>
-          <t>08:00:00</t>
-        </is>
-      </c>
-      <c r="G249" s="9" t="n">
         <v>720</v>
       </c>
     </row>

</xml_diff>